<commit_message>
agrega nuevos pactos, corrige incumbencia d21 y agrega incumbencia d2
</commit_message>
<xml_diff>
--- a/Resultados/Pactos.xlsx
+++ b/Resultados/Pactos.xlsx
@@ -8,19 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivan\Desktop\Ivan\Laboral\EstrategiaSur\GitProjects\Proyeccion-electoral-congreso\Resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA067B5-6CAD-456F-9712-B7C8E36C86FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264DFA02-CDA4-44BB-A2C4-F2834327D196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1665" windowWidth="29040" windowHeight="15720" xr2:uid="{95F9DA68-DEBC-4B6D-8C8C-D1F5C4B96E3B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="6" xr2:uid="{95F9DA68-DEBC-4B6D-8C8C-D1F5C4B96E3B}"/>
   </bookViews>
   <sheets>
     <sheet name="EscConv" sheetId="1" r:id="rId1"/>
     <sheet name="EscCons" sheetId="2" r:id="rId2"/>
     <sheet name="EscMun" sheetId="3" r:id="rId3"/>
+    <sheet name="EscPers1_CHV+" sheetId="4" r:id="rId4"/>
+    <sheet name="EscPers1_CHV" sheetId="5" r:id="rId5"/>
+    <sheet name="EscPers2_CHV+" sheetId="6" r:id="rId6"/>
+    <sheet name="EscPers2_CHV" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">EscCons!$B$2:$C$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EscConv!$B$2:$C$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">EscMun!$B$2:$C$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">EscPers1_CHV!$B$2:$C$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EscPers1_CHV+'!$B$2:$C$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">EscPers2_CHV!$B$2:$C$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'EscPers2_CHV+'!$B$2:$C$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="53">
   <si>
     <t>FA</t>
   </si>
@@ -184,6 +192,24 @@
   </si>
   <si>
     <t>Pactos a concejales de la última elección municipal.</t>
+  </si>
+  <si>
+    <t>Personalizado 1 CHV+</t>
+  </si>
+  <si>
+    <t>Pacto creado a criterio experto donde Amarillos y democratas van en pacto con CHV</t>
+  </si>
+  <si>
+    <t>Personalizado 1 CHV</t>
+  </si>
+  <si>
+    <t>Pacto creado a criterio experto donde Amarillos y democratas van en pacto separado con CHV</t>
+  </si>
+  <si>
+    <t>Personalizado 2 CHV+</t>
+  </si>
+  <si>
+    <t>Personalizado 2 CHV</t>
   </si>
 </sst>
 </file>
@@ -403,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -437,11 +463,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="82">
+  <dxfs count="185">
     <dxf>
       <fill>
         <patternFill>
@@ -483,6 +510,810 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7E350E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFADADAD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2CEEF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -595,6 +1426,44 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -643,6 +1512,344 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
           <bgColor rgb="FF000000"/>
@@ -653,398 +1860,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF7030A0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF7030A0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF00B050"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF00B050"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF7E350E"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF7E350E"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFADADAD"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFADADAD"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2CEEF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2CEEF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAF2D0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDAF2D0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF94DCF8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF94DCF8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFABAB"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFABAB"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1229,6 +2044,226 @@
         <a:xfrm>
           <a:off x="2730500" y="4768850"/>
           <a:ext cx="1676506" cy="942975"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>92075</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1006581</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>736600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D98843F2-1514-4EE5-9F76-DCAAE22CF882}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2733675" y="4851400"/>
+          <a:ext cx="1676506" cy="857250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>92075</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1006581</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>736600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90302903-E49F-49CC-88E7-7C05013F4D7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2733675" y="4851400"/>
+          <a:ext cx="1676506" cy="857250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>92075</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1006581</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>736600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCFB9F7C-4AC4-4CEE-882C-36F87152E623}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2733675" y="4851400"/>
+          <a:ext cx="1676506" cy="857250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>92075</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1006581</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>736600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2996E4D-055C-45BA-B91E-FC0F50856D30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2733675" y="4851400"/>
+          <a:ext cx="1676506" cy="857250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1775,29 +2810,29 @@
   </sheetData>
   <autoFilter ref="B2:C2" xr:uid="{DED54A05-654A-4DD0-A625-003E7E205AB3}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
-      <sortCondition sortBy="cellColor" ref="C2" dxfId="81"/>
+      <sortCondition sortBy="cellColor" ref="C2" dxfId="184"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="B2:C25">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="181" priority="1" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="3" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="179" priority="4" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="5" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="177" priority="6" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="7" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="8" operator="equal">
       <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2026,32 +3061,32 @@
   </sheetData>
   <autoFilter ref="B2:C2" xr:uid="{30C24D76-6A46-4A20-99E0-C96484E3A12C}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
-      <sortCondition sortBy="cellColor" ref="C2" dxfId="79"/>
+      <sortCondition sortBy="cellColor" ref="C2" dxfId="183"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="B2:C25">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="1" operator="equal">
       <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="173" priority="2" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="172" priority="3" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="4" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="5" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="6" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="7" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="8" operator="equal">
       <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2271,7 +3306,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:3" ht="58" x14ac:dyDescent="0.35">
       <c r="B28" s="18" t="s">
         <v>45</v>
       </c>
@@ -2282,50 +3317,1142 @@
   </sheetData>
   <autoFilter ref="B2:C25" xr:uid="{B53DDAD8-76D2-494B-9FFC-BFDFE9B6F19A}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
-      <sortCondition sortBy="cellColor" ref="C2:C25" dxfId="35"/>
+      <sortCondition sortBy="cellColor" ref="C2:C25" dxfId="182"/>
     </sortState>
   </autoFilter>
+  <conditionalFormatting sqref="B2:C25">
+    <cfRule type="cellIs" dxfId="166" priority="1" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="165" priority="2" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="164" priority="3" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="163" priority="4" operator="equal">
+      <formula>"p10"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="162" priority="5" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C3:C25">
-    <cfRule type="cellIs" dxfId="12" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="6" operator="equal">
       <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="160" priority="7" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="8" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="9" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="157" priority="10" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="11" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="12" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="154" priority="13" operator="equal">
       <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A09CB69-558B-4DF2-854D-4D1650AE2035}">
+  <dimension ref="B2:C28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" customWidth="1"/>
+    <col min="5" max="5" width="43.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B15" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B23" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B24" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B27" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="87" x14ac:dyDescent="0.35">
+      <c r="B28" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:C25" xr:uid="{B53DDAD8-76D2-494B-9FFC-BFDFE9B6F19A}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
+      <sortCondition sortBy="cellColor" ref="C2:C25" dxfId="91"/>
+    </sortState>
+  </autoFilter>
   <conditionalFormatting sqref="B2:C25">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="153" priority="1" operator="equal">
       <formula>"p13"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="152" priority="2" operator="equal">
       <formula>"p12"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="3" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="4" operator="equal">
       <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="149" priority="5" operator="equal">
       <formula>"p9"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C25">
+    <cfRule type="cellIs" dxfId="148" priority="6" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="147" priority="7" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="146" priority="8" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="145" priority="9" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="144" priority="10" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="143" priority="11" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="142" priority="12" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="141" priority="13" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4FC4B7E-AE39-4FA8-9CEF-41E9DB92770B}">
+  <dimension ref="B2:C28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" customWidth="1"/>
+    <col min="5" max="5" width="43.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B23" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B24" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B27" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="B28" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:C25" xr:uid="{B53DDAD8-76D2-494B-9FFC-BFDFE9B6F19A}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
+      <sortCondition sortBy="cellColor" ref="C2:C25" dxfId="72"/>
+    </sortState>
+  </autoFilter>
+  <conditionalFormatting sqref="B2:C25">
+    <cfRule type="cellIs" dxfId="140" priority="1" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="139" priority="2" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="3" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="137" priority="4" operator="equal">
+      <formula>"p10"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="5" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C25">
+    <cfRule type="cellIs" dxfId="135" priority="6" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="134" priority="7" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="8" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="9" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="131" priority="10" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="11" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="129" priority="12" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="128" priority="13" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{053AB71A-9767-4372-9388-C06F8B74E6C1}">
+  <dimension ref="B2:C28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" customWidth="1"/>
+    <col min="5" max="5" width="43.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B15" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B23" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B24" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B27" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="87" x14ac:dyDescent="0.35">
+      <c r="B28" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:C25" xr:uid="{B53DDAD8-76D2-494B-9FFC-BFDFE9B6F19A}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
+      <sortCondition sortBy="cellColor" ref="C2:C25" dxfId="55"/>
+    </sortState>
+  </autoFilter>
+  <conditionalFormatting sqref="B2:C25">
+    <cfRule type="cellIs" dxfId="127" priority="1" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="126" priority="2" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="125" priority="3" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="4" operator="equal">
+      <formula>"p10"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="5" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C25">
+    <cfRule type="cellIs" dxfId="122" priority="6" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="121" priority="7" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="8" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="119" priority="9" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="10" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="117" priority="11" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="116" priority="12" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="13" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F421056-ABE0-4205-AB95-533FE69D7C71}">
+  <dimension ref="B2:C28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" customWidth="1"/>
+    <col min="5" max="5" width="43.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B23" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B24" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B27" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="B28" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:C25" xr:uid="{B53DDAD8-76D2-494B-9FFC-BFDFE9B6F19A}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:C25">
+      <sortCondition sortBy="cellColor" ref="C2:C25" dxfId="21"/>
+    </sortState>
+  </autoFilter>
+  <conditionalFormatting sqref="B2:C25">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+      <formula>"p10"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C25">
+    <cfRule type="cellIs" dxfId="114" priority="6" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="113" priority="7" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="112" priority="8" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="9" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="110" priority="10" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="11" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="108" priority="12" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="107" priority="13" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>